<commit_message>
feat(finance): sistema de recuperacao de vendas via Resend email e tooltips explicativas (i) de GMV e Escrow
</commit_message>
<xml_diff>
--- a/docs/diag/env_configuracoes.xlsx
+++ b/docs/diag/env_configuracoes.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -635,7 +635,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>pk_t••••••••zqg6</t>
+          <t>pk_l••••••••Yoz9</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -662,22 +662,22 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>VITE_APP_URL</t>
+          <t>STRIPE_SECRET_KEY</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>http://localhost:5173</t>
+          <t>sk_l••••••••zr6A</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Frontend (Público)</t>
+          <t>Backend (Servidor/Secret)</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim (Protegido)</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>APP_URL</t>
+          <t>VITE_APP_URL</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Backend (Servidor/Secret)</t>
+          <t>Frontend (Público)</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -721,17 +721,17 @@
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>- GitHub Secrets: SUPABASE_SERVICE_ROLE_KEY, SUPABASE_ACCESS_TOKEN, STRIPE_SECRET_KEY</t>
+          <t>e GitHub Actions secrets.</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>SUPABASE_ACCESS_TOKEN</t>
+          <t>APP_URL</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>sbp_••••••••7ba6</t>
+          <t>http://localhost:5173</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Sim (Protegido)</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -758,12 +758,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>SUPABASE_SERVICE_ROLE_KEY</t>
+          <t>SUPABASE_ACCESS_TOKEN</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>sb_s••••••••ggsr</t>
+          <t>sbp_••••••••7ba6</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -790,12 +790,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>REPLICATE_API_KEY</t>
+          <t>SUPABASE_SERVICE_ROLE_KEY</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>r8_c••••••••cZ24</t>
+          <t>sb_s••••••••ggsr</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -822,12 +822,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>GEMINI_API_KEY</t>
+          <t>REPLICATE_API_KEY</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>AQ.A••••••••eBFQ</t>
+          <t>r8_c••••••••cZ24</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -854,17 +854,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>VITE_OPENROUTER_API_KEY</t>
+          <t>GEMINI_API_KEY</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>sk-o••••••••6034</t>
+          <t>AQ.A••••••••eBFQ</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Frontend (Público)</t>
+          <t>Backend (Servidor/Secret)</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -881,27 +881,27 @@
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Google OAuth (supabase)</t>
+          <t>- GitHub Secrets: SUPABASE_SERVICE_ROLE_KEY, SUPABASE_ACCESS_TOKEN, STRIPE_SECRET_KEY</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>GOOGLE_CLIENT_ID</t>
+          <t>VITE_OPENROUTER_API_KEY</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>618628258891-0k11mbjiuv3lrg8gsjlldv6p4qg1p06b.apps.googleusercontent.com</t>
+          <t>sk-o••••••••6034</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Backend (Servidor/Secret)</t>
+          <t>Frontend (Público)</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim (Protegido)</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -918,12 +918,12 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>GOOGLE_CLIENT_SECRET</t>
+          <t>GOOGLE_CLIENT_ID</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>GOCS••••••••Rz4x</t>
+          <t>618628258891-0k11mbjiuv3lrg8gsjlldv6p4qg1p06b.apps.googleusercontent.com</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -933,7 +933,7 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Sim (Protegido)</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -945,27 +945,27 @@
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Upstash Redis (cache)</t>
+          <t>Google OAuth (supabase)</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>VITE_UPSTASH_REDIS_REST_URL</t>
+          <t>GOOGLE_CLIENT_SECRET</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>https://cunning-civet-138870.upstash.io</t>
+          <t>GOCS••••••••Rz4x</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Frontend (Público)</t>
+          <t>Backend (Servidor/Secret)</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim (Protegido)</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -982,12 +982,12 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>VITE_UPSTASH_REDIS_REST_TOKEN</t>
+          <t>VITE_UPSTASH_REDIS_REST_URL</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>gQAA••••••••Q0Yg</t>
+          <t>https://cunning-civet-138870.upstash.io</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -997,7 +997,7 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>Sim (Protegido)</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -1009,27 +1009,27 @@
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Dados de Acesso VPS (Ollama &amp; Tunnel)</t>
+          <t>Upstash Redis (cache)</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>VPS_IP</t>
+          <t>VITE_UPSTASH_REDIS_REST_TOKEN</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>201.46.120.192</t>
+          <t>gQAA••••••••Q0Yg</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Backend (Servidor/Secret)</t>
+          <t>Frontend (Público)</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim (Protegido)</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -1046,12 +1046,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>VPS_SSH_USER</t>
+          <t>VPS_IP</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>root</t>
+          <t>201.46.120.192</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -1078,12 +1078,12 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>VPS_SSH_PORT</t>
+          <t>VPS_SSH_USER</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>6985</t>
+          <t>root</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -1110,12 +1110,12 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>VPS_SSH_PASSWORD</t>
+          <t>VPS_SSH_PORT</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>••••••••</t>
+          <t>6985</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Sim (Protegido)</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -1137,27 +1137,27 @@
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>⚠️ ADICIONE ESSAS DUAS CHAVES NA VERCEL:</t>
+          <t>Dados de Acesso VPS (Ollama &amp; Tunnel)</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>VITE_OLLAMA_API_URL</t>
+          <t>VPS_SSH_PASSWORD</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>http://201.46.120.192/api/chat</t>
+          <t>••••••••</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Frontend (Público)</t>
+          <t>Backend (Servidor/Secret)</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim (Protegido)</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -1174,12 +1174,12 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>VITE_OLLAMA_API_AUTH</t>
+          <t>VITE_OLLAMA_API_URL</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Basi••••••••OTE4</t>
+          <t>http://201.46.120.192/api/chat</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Sim (Protegido)</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -1201,22 +1201,22 @@
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Ngrok Token para o Colab AI Server</t>
+          <t>⚠️ ADICIONE ESSAS DUAS CHAVES NA VERCEL:</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>NGROK_AUTH_TOKEN</t>
+          <t>VITE_OLLAMA_API_AUTH</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>3GBR••••••••8g4G</t>
+          <t>Basi••••••••OTE4</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Backend (Servidor/Secret)</t>
+          <t>Frontend (Público)</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -1233,30 +1233,62 @@
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
+          <t>Ngrok Token para o Colab AI Server</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>NGROK_AUTH_TOKEN</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>3GBR••••••••8g4G</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Backend (Servidor/Secret)</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Sim (Protegido)</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Configurado</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
           <t>Configuração de Métodos de Pagamento do Stripe (Japão: Konbini, Apple Pay, Google Pay)</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>VITE_STRIPE_PAYMENT_METHOD_CONFIG_ID</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>pmc_1O8JCnHLdM</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>Frontend (Público)</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
+      <c r="F27" s="8" t="inlineStr">
         <is>
           <t>Configurado</t>
         </is>

</xml_diff>